<commit_message>
feat(concierge): coherent buyer experience + per-county delivery
- /welcome: rewrite from API/SaaS onboarding (API keys, webhooks, team
  invites) to the concierge reality — a weekly lead list by email
- /dashboard: honest preview banner (email delivery today; live dashboard
  on the roadmap), CTA -> /pricing
- build-lead-list.mjs: optional county arg for single-county subscribers
- make-xlsx.py: banner adapts to the counties actually in the list
- first-dollar-playbook.md: post-payment welcome email + tightened weekly
  delivery SOP (live re-fetch + county arg)
- refresh South-FL lead sample (filed 2026-06-05..16)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/validation/south-fl-new-liquor-leads.xlsx
+++ b/validation/south-fl-new-liquor-leads.xlsx
@@ -561,7 +561,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sample lead list · 25 brand-new venues licensed to serve alcohol (Broward / Miami-Dade / Palm Beach) · filed 2026-06-01 to 2026-06-12</t>
+          <t>Sample lead list · 25 brand-new venues licensed to serve alcohol (Broward / Miami-Dade / Palm Beach) · filed 2026-06-05 to 2026-06-16</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Mandarin Feast INC</t>
+          <t>Soctainer</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -647,50 +647,48 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>BEV6019358</t>
+          <t>BEV2339051</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>6619 Boynton Beach Blvd</t>
+          <t>820 SW 20 Ave</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Boynton Beach</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Palm Beach</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>33437</t>
+          <t>33135</t>
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>46185</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v>46477</v>
-      </c>
+        <v>46189</v>
+      </c>
+      <c r="J6" s="6" t="inlineStr"/>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>Mandarin Feast INC</t>
+          <t>Soccer 8 LLC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Sylvain's Cafe</t>
+          <t>Burt &amp; Maxs Bar &amp; Grille</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Beer &amp; wine, on premises</t>
+          <t>Full liquor (quota), on/off premises</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -700,48 +698,48 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>BEV1625326</t>
+          <t>BEV6016081</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>1634 SE 3rd Ct</t>
+          <t>9089 West Atlantic Avenue, Suite 100</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Deerfield Beach</t>
+          <t>Delray Beach</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Broward</t>
+          <t>Palm Beach</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>33441</t>
+          <t>33446</t>
         </is>
       </c>
       <c r="I7" s="10" t="n">
-        <v>46185</v>
+        <v>46189</v>
       </c>
       <c r="J7" s="9" t="inlineStr"/>
       <c r="K7" s="8" t="inlineStr">
         <is>
-          <t>Cube Holdings LLC</t>
+          <t>Shv1 LLC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Bar Restaurant Urbano Hollywood</t>
+          <t>G's Kitchen &amp; Bar</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -751,17 +749,17 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>BEV1606920</t>
+          <t>BEV1625329</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>2020 Hollywood Blvd</t>
+          <t>4877 Coconut Creek Pkwy, Store #28</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Hollywood</t>
+          <t>Margate</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -771,28 +769,28 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>33020</t>
+          <t>33063</t>
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>46184</v>
+        <v>46189</v>
       </c>
       <c r="J8" s="6" t="inlineStr"/>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>Bar Resturant Urbano LLC</t>
+          <t>Lacer Trading LLC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>John G's</t>
+          <t>Daniella's At Village Walk</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -802,17 +800,17 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>BEV6018638</t>
+          <t>BEV6019360</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>264 S Ocean Blvd</t>
+          <t>2540 Villagewalk Circle, Suite 3</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Manalapan</t>
+          <t>Wellington</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -822,23 +820,23 @@
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>33462</t>
+          <t>33414</t>
         </is>
       </c>
       <c r="I9" s="10" t="n">
-        <v>46184</v>
+        <v>46189</v>
       </c>
       <c r="J9" s="9" t="inlineStr"/>
       <c r="K9" s="8" t="inlineStr">
         <is>
-          <t>Sikellis Investments LLC</t>
+          <t>Pb Food &amp; Supply Distributors LLC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Whiskey Tango Bar &amp; Grill</t>
+          <t>Sauce 'em</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -853,43 +851,43 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>BEV6000346</t>
+          <t>BEV1625328</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>1306 N Military Trail</t>
+          <t>123 NE 20th Avenue, Bay 17</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>West Palm Beach</t>
+          <t>Deerfield Beach</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Palm Beach</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>33409</t>
+          <t>33441</t>
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>46184</v>
+        <v>46189</v>
       </c>
       <c r="J10" s="6" t="inlineStr"/>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>Eazy Hospitality LLC</t>
+          <t>Sauce 'em LLC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Oregano Greek Kitchen</t>
+          <t>Replay Club</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -904,45 +902,45 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>BEV2339045</t>
+          <t>BEV6019359</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>15356 NW 79th Ct</t>
+          <t>7700 High Ridge Road</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Miami Lakes</t>
+          <t>Boynton Beach</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Palm Beach</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>33016</t>
+          <t>33426</t>
         </is>
       </c>
       <c r="I11" s="10" t="n">
-        <v>46183</v>
+        <v>46188</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46477</v>
       </c>
       <c r="K11" s="8" t="inlineStr">
         <is>
-          <t>Oregano Greek Kitchen</t>
+          <t>Rally Club LLC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Skippy's Pizza</t>
+          <t>Maestro Italian Bakery</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -957,48 +955,48 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>BEV1625325</t>
+          <t>BEV2339049</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>2720 E Oakland Park Blvd, Ste 104</t>
+          <t>3067 NE 163rd Street</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Fort Lauderdale</t>
+          <t>North Miami Beach</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Broward</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>33306</t>
+          <t>33160</t>
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>46183</v>
+        <v>46188</v>
       </c>
       <c r="J12" s="6" t="inlineStr"/>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>1 Big G Enterprise LLC</t>
+          <t>Masterone LLC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Marthas Wine Bar</t>
+          <t>Shamama Restaurant</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Beer &amp; wine, on premises</t>
+          <t>Full liquor (quota), on/off premises</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -1008,50 +1006,48 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>BEV6019356</t>
+          <t>BEV1625327</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>509 Park Place</t>
+          <t>7456 Royal Palm Blvd</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>West Palm Beach</t>
+          <t>Margate</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Palm Beach</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>33401</t>
+          <t>33063</t>
         </is>
       </c>
       <c r="I13" s="10" t="n">
-        <v>46182</v>
-      </c>
-      <c r="J13" s="10" t="n">
-        <v>46477</v>
-      </c>
+        <v>46188</v>
+      </c>
+      <c r="J13" s="9" t="inlineStr"/>
       <c r="K13" s="8" t="inlineStr">
         <is>
-          <t>Evernia Wine Bar LLC</t>
+          <t>Shamama Restaurant, INC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Basilico Coral Gables</t>
+          <t>Viaoeste Cafe And Bakery Doral LLC</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1061,17 +1057,17 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>BEV2335859</t>
+          <t>BEV2339046</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>2312 Ponce De Leon Blvd</t>
+          <t>11150 NW 82nd Street, Unit 103</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Coral Gables</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1081,23 +1077,23 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>33134</t>
+          <t>33178</t>
         </is>
       </c>
       <c r="I14" s="7" t="n">
-        <v>46182</v>
+        <v>46188</v>
       </c>
       <c r="J14" s="6" t="inlineStr"/>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>Basilico Coral Gables INC.</t>
+          <t>Viaoeste Cafe And Bakery Doral LLC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Origen</t>
+          <t>Sulta Rosa</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -1112,48 +1108,48 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>BEV1625322</t>
+          <t>BEV2339047</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>10000 Stirling Rd Suite 8</t>
+          <t>821 Lincoln Rd</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>Cooper City</t>
+          <t>Miami Beach</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>Broward</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>33024</t>
+          <t>33139</t>
         </is>
       </c>
       <c r="I15" s="10" t="n">
-        <v>46182</v>
+        <v>46188</v>
       </c>
       <c r="J15" s="9" t="inlineStr"/>
       <c r="K15" s="8" t="inlineStr">
         <is>
-          <t>International Gastronomic Development LLC</t>
+          <t>Sulta Rosa INC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>La Condesa Mexican Restaurant</t>
+          <t>Mandarin Feast INC</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -1163,48 +1159,48 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>BEV1625323</t>
+          <t>BEV6019358</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>1800 Bell Tower Lane</t>
+          <t>6619 Boynton Beach Blvd</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Weston</t>
+          <t>Boynton Beach</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Broward</t>
+          <t>Palm Beach</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>33326</t>
+          <t>33437</t>
         </is>
       </c>
       <c r="I16" s="7" t="n">
-        <v>46182</v>
+        <v>46185</v>
       </c>
       <c r="J16" s="6" t="inlineStr"/>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>J &amp; S Restaurants LLC</t>
+          <t>Mandarin Feast INC</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Gary Racks Farmhouse Kitchen</t>
+          <t>Sylvain's Cafe</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -1214,17 +1210,17 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>BEV1625324</t>
+          <t>BEV1625326</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>3314 University Drive, Unit 13 And Unit 14</t>
+          <t>1634 SE 3rd Ct</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>Coral Springs</t>
+          <t>Deerfield Beach</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
@@ -1234,28 +1230,28 @@
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>33065</t>
+          <t>33441</t>
         </is>
       </c>
       <c r="I17" s="10" t="n">
-        <v>46182</v>
+        <v>46185</v>
       </c>
       <c r="J17" s="9" t="inlineStr"/>
       <c r="K17" s="8" t="inlineStr">
         <is>
-          <t>G&amp;V5 LLC</t>
+          <t>Cube Holdings LLC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Sushi Sake South Miami</t>
+          <t>Bar Restaurant Urbano Hollywood</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Beer &amp; wine, on premises</t>
+          <t>Full liquor (quota), on/off premises</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -1265,43 +1261,43 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>BEV2339044</t>
+          <t>BEV1606920</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>5829 SW 73 St, #5b</t>
+          <t>2020 Hollywood Blvd</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>South Miami</t>
+          <t>Hollywood</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>33143</t>
+          <t>33020</t>
         </is>
       </c>
       <c r="I18" s="7" t="n">
-        <v>46181</v>
+        <v>46184</v>
       </c>
       <c r="J18" s="6" t="inlineStr"/>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>Ss South Miami LLC</t>
+          <t>Bar Resturant Urbano Hollywood LLC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>La Traila BBQ</t>
+          <t>John G's</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -1316,48 +1312,48 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>BEV2339041</t>
+          <t>BEV6018638</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>5840 SW 71st Street, B</t>
+          <t>264 S Ocean Blvd</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>South Miami</t>
+          <t>Manalapan</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Palm Beach</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>33143</t>
+          <t>33462</t>
         </is>
       </c>
       <c r="I19" s="10" t="n">
-        <v>46178</v>
+        <v>46184</v>
       </c>
       <c r="J19" s="9" t="inlineStr"/>
       <c r="K19" s="8" t="inlineStr">
         <is>
-          <t>La Traila BBQ LLC</t>
+          <t>Sikellis Investments LLC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Lucky 9 Bartending &amp; Consulting</t>
+          <t>Whiskey Tango Bar &amp; Grill</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Catering</t>
+          <t>Full liquor (quota), on/off premises</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -1367,45 +1363,43 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>BEV2339040</t>
+          <t>BEV6000346</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>528 SW 9 Ave</t>
+          <t>1306 N Military Trail</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>West Palm Beach</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Palm Beach</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>33130</t>
+          <t>33409</t>
         </is>
       </c>
       <c r="I20" s="7" t="n">
-        <v>46178</v>
-      </c>
-      <c r="J20" s="7" t="n">
-        <v>46477</v>
-      </c>
+        <v>46184</v>
+      </c>
+      <c r="J20" s="6" t="inlineStr"/>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>Lucky 9 Bartending &amp; Consulting INC</t>
+          <t>Eazy Hospitality LLC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Park Grove Bistro</t>
+          <t>Oregano Greek Kitchen</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -1420,17 +1414,17 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>BEV2339038</t>
+          <t>BEV2339045</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>2821 South Bayshore Drive, #300</t>
+          <t>15356 NW 79th Ct</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Miami Lakes</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
@@ -1440,30 +1434,30 @@
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>33133</t>
+          <t>33016</t>
         </is>
       </c>
       <c r="I21" s="10" t="n">
-        <v>46178</v>
+        <v>46183</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46477</v>
       </c>
       <c r="K21" s="8" t="inlineStr">
         <is>
-          <t>Park Grove Bistro INC</t>
+          <t>Oregano Greek Kitchen</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Lucca Modern Trattoria Rustic Soul</t>
+          <t>Skippy's Pizza</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -1473,43 +1467,43 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>BEV2339039</t>
+          <t>BEV1625325</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>7450 NW 104th Avenue, Suite C106</t>
+          <t>2720 E Oakland Park Blvd, Ste 104</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Doral</t>
+          <t>Fort Lauderdale</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>33178</t>
+          <t>33306</t>
         </is>
       </c>
       <c r="I22" s="7" t="n">
-        <v>46178</v>
+        <v>46183</v>
       </c>
       <c r="J22" s="6" t="inlineStr"/>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>Cm Italian Gourmet LLC</t>
+          <t>1 Big G Enterprise LLC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Low Key Kava</t>
+          <t>Marthas Wine Bar</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -1524,12 +1518,12 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>BEV6019355</t>
+          <t>BEV6019356</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>404 S Military Trail</t>
+          <t>509 Park Place</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1544,23 +1538,25 @@
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>33415</t>
+          <t>33401</t>
         </is>
       </c>
       <c r="I23" s="10" t="n">
-        <v>46177</v>
-      </c>
-      <c r="J23" s="9" t="inlineStr"/>
+        <v>46182</v>
+      </c>
+      <c r="J23" s="10" t="n">
+        <v>46477</v>
+      </c>
       <c r="K23" s="8" t="inlineStr">
         <is>
-          <t>404 Kava LLC</t>
+          <t>Evernia Wine Bar LLC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Singing Bamboo</t>
+          <t>Basilico Coral Gables</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -1575,48 +1571,48 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>BEV6003318</t>
+          <t>BEV2335859</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>2845 N Militar Trail Suites 11-15</t>
+          <t>2312 Ponce De Leon Blvd</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>West Palm Beach</t>
+          <t>Coral Gables</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Palm Beach</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>33409</t>
+          <t>33134</t>
         </is>
       </c>
       <c r="I24" s="7" t="n">
-        <v>46177</v>
+        <v>46182</v>
       </c>
       <c r="J24" s="6" t="inlineStr"/>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>Cqd Dragon 1 LLC</t>
+          <t>Basilico Coral Gables INC.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Ford's Garage</t>
+          <t>Origen</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -1626,48 +1622,48 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>BEV6019354</t>
+          <t>BEV1625322</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>365 N Congress Ave</t>
+          <t>10000 Stirling Rd Suite 8</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>Boynton Beach</t>
+          <t>Cooper City</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>Palm Beach</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>33426</t>
+          <t>33024</t>
         </is>
       </c>
       <c r="I25" s="10" t="n">
-        <v>46177</v>
+        <v>46182</v>
       </c>
       <c r="J25" s="9" t="inlineStr"/>
       <c r="K25" s="8" t="inlineStr">
         <is>
-          <t>Ford's Garage Boynton Beach, LLC</t>
+          <t>International Gastronomic Development LLC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Rivalries Sports Pub</t>
+          <t>La Condesa Mexican Restaurant</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Beer &amp; wine, on premises</t>
+          <t>Full liquor (quota), on/off premises</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -1677,45 +1673,43 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>BEV6019352</t>
+          <t>BEV1625323</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>510 East Ocean Avenue, 101</t>
+          <t>1800 Bell Tower Lane</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Boynton Beach</t>
+          <t>Weston</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Palm Beach</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>33435</t>
+          <t>33326</t>
         </is>
       </c>
       <c r="I26" s="7" t="n">
-        <v>46176</v>
-      </c>
-      <c r="J26" s="7" t="n">
-        <v>46477</v>
-      </c>
+        <v>46182</v>
+      </c>
+      <c r="J26" s="6" t="inlineStr"/>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>Mvb, INC</t>
+          <t>J &amp; S Restaurants LLC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Old Lisbon Aventura</t>
+          <t>Gary Racks Farmhouse Kitchen</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -1730,43 +1724,43 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>BEV2334577</t>
+          <t>BEV1625324</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>2960 NE 199th St, #5a</t>
+          <t>3314 University Drive, Unit 13 And Unit 14</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>Aventura</t>
+          <t>Coral Springs</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>33180</t>
+          <t>33065</t>
         </is>
       </c>
       <c r="I27" s="10" t="n">
-        <v>46176</v>
+        <v>46182</v>
       </c>
       <c r="J27" s="9" t="inlineStr"/>
       <c r="K27" s="8" t="inlineStr">
         <is>
-          <t>Old Lisbon Aventura LLC</t>
+          <t>G&amp;V5 LLC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Rio's Cafe &amp; Grill</t>
+          <t>Sushi Sake South Miami</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1781,45 +1775,43 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>BEV1625320</t>
+          <t>BEV2339044</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>3937 N Federal Highway</t>
+          <t>5829 SW 73 St, #5b</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Pompano Beach</t>
+          <t>South Miami</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Broward</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>33064</t>
+          <t>33143</t>
         </is>
       </c>
       <c r="I28" s="7" t="n">
-        <v>46175</v>
-      </c>
-      <c r="J28" s="7" t="n">
-        <v>46477</v>
-      </c>
+        <v>46181</v>
+      </c>
+      <c r="J28" s="6" t="inlineStr"/>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>Rio's Brazilian Meat Market &amp; Grocery, LLC</t>
+          <t>Ss South Miami LLC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Mayfair House Hotel &amp; Garden</t>
+          <t>La Traila BBQ</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -1834,17 +1826,17 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>BEV2333302</t>
+          <t>BEV2339041</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>3000 Florida Avenue</t>
+          <t>5840 SW 71st Street, B</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>South Miami</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
@@ -1854,30 +1846,28 @@
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>33133</t>
+          <t>33143</t>
         </is>
       </c>
       <c r="I29" s="10" t="n">
-        <v>46174</v>
-      </c>
-      <c r="J29" s="10" t="n">
-        <v>46477</v>
-      </c>
+        <v>46178</v>
+      </c>
+      <c r="J29" s="9" t="inlineStr"/>
       <c r="K29" s="8" t="inlineStr">
         <is>
-          <t>Dean Mcg Propco LLC</t>
+          <t>La Traila BBQ LLC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Diadem Pickleball Complex Wellington</t>
+          <t>Lucky 9 Bartending &amp; Consulting</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Beer &amp; wine, on premises</t>
+          <t>Catering</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -1887,38 +1877,38 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>BEV6019351</t>
+          <t>BEV2339040</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>10570 W Forest Hill Blvd</t>
+          <t>528 SW 9 Ave</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Wellington</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Palm Beach</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>33414</t>
+          <t>33130</t>
         </is>
       </c>
       <c r="I30" s="7" t="n">
-        <v>46174</v>
+        <v>46178</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>46477</v>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>Valisi Consultant Corp</t>
+          <t>Lucky 9 Bartending &amp; Consulting INC</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1961,7 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -1991,7 +1981,7 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -2009,7 +1999,7 @@
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -2029,7 +2019,7 @@
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(validation): regenerate June 5–17 sample + log Bellken/Prestige outreach
- regenerated south-fl-new-liquor-leads.{csv,json,xlsx} (25 on-premises venues,
  filed June 5–17, Broward/Miami-Dade/Palm Beach)
- prospect-list.csv: Bellken emailed 2026-06-18; Prestige follow-up sent

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/validation/south-fl-new-liquor-leads.xlsx
+++ b/validation/south-fl-new-liquor-leads.xlsx
@@ -561,7 +561,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sample lead list · 25 brand-new venues licensed to serve alcohol (Broward / Miami-Dade / Palm Beach) · filed 2026-06-05 to 2026-06-16</t>
+          <t>Sample lead list · 25 brand-new venues licensed to serve alcohol (Broward / Miami-Dade / Palm Beach) · filed 2026-06-05 to 2026-06-17</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Soctainer</t>
+          <t>El Patio Del Chef</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -647,48 +647,48 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>BEV2339051</t>
+          <t>BEV1625331</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>820 SW 20 Ave</t>
+          <t>201 N 21st Avenue</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Hollywood</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>33135</t>
+          <t>33020</t>
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="J6" s="6" t="inlineStr"/>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>Soccer 8 LLC</t>
+          <t>Two Brothers Fl LLC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Burt &amp; Maxs Bar &amp; Grille</t>
+          <t>Soctainer</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -698,27 +698,27 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>BEV6016081</t>
+          <t>BEV2339051</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>9089 West Atlantic Avenue, Suite 100</t>
+          <t>820 SW 20 Ave</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Delray Beach</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Palm Beach</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>33446</t>
+          <t>33135</t>
         </is>
       </c>
       <c r="I7" s="10" t="n">
@@ -727,19 +727,19 @@
       <c r="J7" s="9" t="inlineStr"/>
       <c r="K7" s="8" t="inlineStr">
         <is>
-          <t>Shv1 LLC</t>
+          <t>Soccer 8 LLC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>G's Kitchen &amp; Bar</t>
+          <t>Burt &amp; Maxs Bar &amp; Grille</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Beer &amp; wine, on premises</t>
+          <t>Full liquor (quota), on/off premises</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -749,27 +749,27 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>BEV1625329</t>
+          <t>BEV6016081</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>4877 Coconut Creek Pkwy, Store #28</t>
+          <t>9089 West Atlantic Avenue, Suite 100</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Margate</t>
+          <t>Delray Beach</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Broward</t>
+          <t>Palm Beach</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>33063</t>
+          <t>33446</t>
         </is>
       </c>
       <c r="I8" s="7" t="n">
@@ -778,7 +778,7 @@
       <c r="J8" s="6" t="inlineStr"/>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>Lacer Trading LLC</t>
+          <t>Shv1 LLC</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Replay Club</t>
+          <t>G's Kitchen &amp; Bar</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -902,45 +902,43 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>BEV6019359</t>
+          <t>BEV1625329</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>7700 High Ridge Road</t>
+          <t>4877 Coconut Creek Pkwy, Store #28</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Boynton Beach</t>
+          <t>Margate</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Palm Beach</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>33426</t>
+          <t>33063</t>
         </is>
       </c>
       <c r="I11" s="10" t="n">
-        <v>46188</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>46477</v>
-      </c>
+        <v>46189</v>
+      </c>
+      <c r="J11" s="9" t="inlineStr"/>
       <c r="K11" s="8" t="inlineStr">
         <is>
-          <t>Rally Club LLC</t>
+          <t>Lacer Trading LLC</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Maestro Italian Bakery</t>
+          <t>Replay Club</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -955,48 +953,50 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>BEV2339049</t>
+          <t>BEV6019359</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>3067 NE 163rd Street</t>
+          <t>7700 High Ridge Road</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>North Miami Beach</t>
+          <t>Boynton Beach</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Palm Beach</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>33160</t>
+          <t>33426</t>
         </is>
       </c>
       <c r="I12" s="7" t="n">
         <v>46188</v>
       </c>
-      <c r="J12" s="6" t="inlineStr"/>
+      <c r="J12" s="7" t="n">
+        <v>46477</v>
+      </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>Masterone LLC</t>
+          <t>Rally Club LLC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Shamama Restaurant</t>
+          <t>Maestro Italian Bakery</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -1006,27 +1006,27 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>BEV1625327</t>
+          <t>BEV2339049</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>7456 Royal Palm Blvd</t>
+          <t>3067 NE 163rd Street</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>Margate</t>
+          <t>North Miami Beach</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Broward</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>33063</t>
+          <t>33160</t>
         </is>
       </c>
       <c r="I13" s="10" t="n">
@@ -1035,19 +1035,19 @@
       <c r="J13" s="9" t="inlineStr"/>
       <c r="K13" s="8" t="inlineStr">
         <is>
-          <t>Shamama Restaurant, INC</t>
+          <t>Masterone LLC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Viaoeste Cafe And Bakery Doral LLC</t>
+          <t>Shamama Restaurant</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Beer &amp; wine, on premises</t>
+          <t>Full liquor (quota), on/off premises</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -1057,27 +1057,27 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>BEV2339046</t>
+          <t>BEV1625327</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>11150 NW 82nd Street, Unit 103</t>
+          <t>7456 Royal Palm Blvd</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Margate</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>33178</t>
+          <t>33063</t>
         </is>
       </c>
       <c r="I14" s="7" t="n">
@@ -1086,14 +1086,14 @@
       <c r="J14" s="6" t="inlineStr"/>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>Viaoeste Cafe And Bakery Doral LLC</t>
+          <t>Shamama Restaurant, INC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Sulta Rosa</t>
+          <t>Viaoeste Cafe And Bakery Doral LLC</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -1108,17 +1108,17 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>BEV2339047</t>
+          <t>BEV2339046</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>821 Lincoln Rd</t>
+          <t>11150 NW 82nd Street, Unit 103</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>Miami Beach</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>33139</t>
+          <t>33178</t>
         </is>
       </c>
       <c r="I15" s="10" t="n">
@@ -1137,14 +1137,14 @@
       <c r="J15" s="9" t="inlineStr"/>
       <c r="K15" s="8" t="inlineStr">
         <is>
-          <t>Sulta Rosa INC</t>
+          <t>Viaoeste Cafe And Bakery Doral LLC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Mandarin Feast INC</t>
+          <t>Sulta Rosa</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1159,43 +1159,43 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>BEV6019358</t>
+          <t>BEV2339047</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>6619 Boynton Beach Blvd</t>
+          <t>821 Lincoln Rd</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Boynton Beach</t>
+          <t>Miami Beach</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Palm Beach</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>33437</t>
+          <t>33139</t>
         </is>
       </c>
       <c r="I16" s="7" t="n">
-        <v>46185</v>
+        <v>46188</v>
       </c>
       <c r="J16" s="6" t="inlineStr"/>
       <c r="K16" s="5" t="inlineStr">
         <is>
-          <t>Mandarin Feast INC</t>
+          <t>Sulta Rosa INC</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Sylvain's Cafe</t>
+          <t>Mandarin Feast INC</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -1210,27 +1210,27 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>BEV1625326</t>
+          <t>BEV6019358</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>1634 SE 3rd Ct</t>
+          <t>6619 Boynton Beach Blvd</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>Deerfield Beach</t>
+          <t>Boynton Beach</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>Broward</t>
+          <t>Palm Beach</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>33441</t>
+          <t>33437</t>
         </is>
       </c>
       <c r="I17" s="10" t="n">
@@ -1239,19 +1239,19 @@
       <c r="J17" s="9" t="inlineStr"/>
       <c r="K17" s="8" t="inlineStr">
         <is>
-          <t>Cube Holdings LLC</t>
+          <t>Mandarin Feast INC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Bar Restaurant Urbano Hollywood</t>
+          <t>Sylvain's Cafe</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -1261,17 +1261,17 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>BEV1606920</t>
+          <t>BEV1625326</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>2020 Hollywood Blvd</t>
+          <t>1634 SE 3rd Ct</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Hollywood</t>
+          <t>Deerfield Beach</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -1281,23 +1281,23 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>33020</t>
+          <t>33441</t>
         </is>
       </c>
       <c r="I18" s="7" t="n">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="J18" s="6" t="inlineStr"/>
       <c r="K18" s="5" t="inlineStr">
         <is>
-          <t>Bar Resturant Urbano Hollywood LLC</t>
+          <t>Cube Holdings LLC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>John G's</t>
+          <t>Bar Restaurant Urbano Hollywood</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -1312,27 +1312,27 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>BEV6018638</t>
+          <t>BEV1606920</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>264 S Ocean Blvd</t>
+          <t>2020 Hollywood Blvd</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Manalapan</t>
+          <t>Hollywood</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Palm Beach</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>33462</t>
+          <t>33020</t>
         </is>
       </c>
       <c r="I19" s="10" t="n">
@@ -1341,14 +1341,14 @@
       <c r="J19" s="9" t="inlineStr"/>
       <c r="K19" s="8" t="inlineStr">
         <is>
-          <t>Sikellis Investments LLC</t>
+          <t>Bar Resturant Urbano Hollywood LLC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Whiskey Tango Bar &amp; Grill</t>
+          <t>John G's</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1363,17 +1363,17 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>BEV6000346</t>
+          <t>BEV6018638</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>1306 N Military Trail</t>
+          <t>264 S Ocean Blvd</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>West Palm Beach</t>
+          <t>Manalapan</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>33409</t>
+          <t>33462</t>
         </is>
       </c>
       <c r="I20" s="7" t="n">
@@ -1392,19 +1392,19 @@
       <c r="J20" s="6" t="inlineStr"/>
       <c r="K20" s="5" t="inlineStr">
         <is>
-          <t>Eazy Hospitality LLC</t>
+          <t>Sikellis Investments LLC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Oregano Greek Kitchen</t>
+          <t>Whiskey Tango Bar &amp; Grill</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Beer &amp; wine, on premises</t>
+          <t>Full liquor (quota), on/off premises</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -1414,45 +1414,43 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>BEV2339045</t>
+          <t>BEV6000346</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>15356 NW 79th Ct</t>
+          <t>1306 N Military Trail</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Miami Lakes</t>
+          <t>West Palm Beach</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Palm Beach</t>
         </is>
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>33016</t>
+          <t>33409</t>
         </is>
       </c>
       <c r="I21" s="10" t="n">
-        <v>46183</v>
-      </c>
-      <c r="J21" s="10" t="n">
-        <v>46477</v>
-      </c>
+        <v>46184</v>
+      </c>
+      <c r="J21" s="9" t="inlineStr"/>
       <c r="K21" s="8" t="inlineStr">
         <is>
-          <t>Oregano Greek Kitchen</t>
+          <t>Eazy Hospitality LLC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Skippy's Pizza</t>
+          <t>Oregano Greek Kitchen</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1467,43 +1465,45 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>BEV1625325</t>
+          <t>BEV2339045</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>2720 E Oakland Park Blvd, Ste 104</t>
+          <t>15356 NW 79th Ct</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Fort Lauderdale</t>
+          <t>Miami Lakes</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Broward</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>33306</t>
+          <t>33016</t>
         </is>
       </c>
       <c r="I22" s="7" t="n">
         <v>46183</v>
       </c>
-      <c r="J22" s="6" t="inlineStr"/>
+      <c r="J22" s="7" t="n">
+        <v>46477</v>
+      </c>
       <c r="K22" s="5" t="inlineStr">
         <is>
-          <t>1 Big G Enterprise LLC</t>
+          <t>Oregano Greek Kitchen</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Marthas Wine Bar</t>
+          <t>Skippy's Pizza</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
@@ -1518,50 +1518,48 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>BEV6019356</t>
+          <t>BEV1625325</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>509 Park Place</t>
+          <t>2720 E Oakland Park Blvd, Ste 104</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>West Palm Beach</t>
+          <t>Fort Lauderdale</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>Palm Beach</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>33401</t>
+          <t>33306</t>
         </is>
       </c>
       <c r="I23" s="10" t="n">
-        <v>46182</v>
-      </c>
-      <c r="J23" s="10" t="n">
-        <v>46477</v>
-      </c>
+        <v>46183</v>
+      </c>
+      <c r="J23" s="9" t="inlineStr"/>
       <c r="K23" s="8" t="inlineStr">
         <is>
-          <t>Evernia Wine Bar LLC</t>
+          <t>1 Big G Enterprise LLC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Basilico Coral Gables</t>
+          <t>Marthas Wine Bar</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -1571,48 +1569,50 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>BEV2335859</t>
+          <t>BEV6019356</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>2312 Ponce De Leon Blvd</t>
+          <t>509 Park Place</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Coral Gables</t>
+          <t>West Palm Beach</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Palm Beach</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>33134</t>
+          <t>33401</t>
         </is>
       </c>
       <c r="I24" s="7" t="n">
         <v>46182</v>
       </c>
-      <c r="J24" s="6" t="inlineStr"/>
+      <c r="J24" s="7" t="n">
+        <v>46477</v>
+      </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>Basilico Coral Gables INC.</t>
+          <t>Evernia Wine Bar LLC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Origen</t>
+          <t>Basilico Coral Gables</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Beer &amp; wine, on premises</t>
+          <t>Full liquor (quota), on/off premises</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -1622,27 +1622,27 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>BEV1625322</t>
+          <t>BEV2335859</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>10000 Stirling Rd Suite 8</t>
+          <t>2312 Ponce De Leon Blvd</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>Cooper City</t>
+          <t>Coral Gables</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>Broward</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>33024</t>
+          <t>33134</t>
         </is>
       </c>
       <c r="I25" s="10" t="n">
@@ -1651,19 +1651,19 @@
       <c r="J25" s="9" t="inlineStr"/>
       <c r="K25" s="8" t="inlineStr">
         <is>
-          <t>International Gastronomic Development LLC</t>
+          <t>Basilico Coral Gables INC.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>La Condesa Mexican Restaurant</t>
+          <t>Origen</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -1673,17 +1673,17 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>BEV1625323</t>
+          <t>BEV1625322</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>1800 Bell Tower Lane</t>
+          <t>10000 Stirling Rd Suite 8</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Weston</t>
+          <t>Cooper City</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>33326</t>
+          <t>33024</t>
         </is>
       </c>
       <c r="I26" s="7" t="n">
@@ -1702,14 +1702,14 @@
       <c r="J26" s="6" t="inlineStr"/>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>J &amp; S Restaurants LLC</t>
+          <t>International Gastronomic Development LLC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Gary Racks Farmhouse Kitchen</t>
+          <t>La Condesa Mexican Restaurant</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -1724,17 +1724,17 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>BEV1625324</t>
+          <t>BEV1625323</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>3314 University Drive, Unit 13 And Unit 14</t>
+          <t>1800 Bell Tower Lane</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>Coral Springs</t>
+          <t>Weston</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>33065</t>
+          <t>33326</t>
         </is>
       </c>
       <c r="I27" s="10" t="n">
@@ -1753,19 +1753,19 @@
       <c r="J27" s="9" t="inlineStr"/>
       <c r="K27" s="8" t="inlineStr">
         <is>
-          <t>G&amp;V5 LLC</t>
+          <t>J &amp; S Restaurants LLC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Sushi Sake South Miami</t>
+          <t>Gary Racks Farmhouse Kitchen</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Beer &amp; wine, on premises</t>
+          <t>Full liquor (quota), on/off premises</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -1775,48 +1775,48 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>BEV2339044</t>
+          <t>BEV1625324</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>5829 SW 73 St, #5b</t>
+          <t>3314 University Drive, Unit 13 And Unit 14</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>South Miami</t>
+          <t>Coral Springs</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Broward</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>33143</t>
+          <t>33065</t>
         </is>
       </c>
       <c r="I28" s="7" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="J28" s="6" t="inlineStr"/>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>Ss South Miami LLC</t>
+          <t>G&amp;V5 LLC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>La Traila BBQ</t>
+          <t>Sushi Sake South Miami</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Full liquor (quota), on/off premises</t>
+          <t>Beer &amp; wine, on premises</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -1826,12 +1826,12 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>BEV2339041</t>
+          <t>BEV2339044</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>5840 SW 71st Street, B</t>
+          <t>5829 SW 73 St, #5b</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -1850,24 +1850,24 @@
         </is>
       </c>
       <c r="I29" s="10" t="n">
-        <v>46178</v>
+        <v>46181</v>
       </c>
       <c r="J29" s="9" t="inlineStr"/>
       <c r="K29" s="8" t="inlineStr">
         <is>
-          <t>La Traila BBQ LLC</t>
+          <t>Ss South Miami LLC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Lucky 9 Bartending &amp; Consulting</t>
+          <t>La Traila BBQ</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Catering</t>
+          <t>Full liquor (quota), on/off premises</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -1877,17 +1877,17 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>BEV2339040</t>
+          <t>BEV2339041</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>528 SW 9 Ave</t>
+          <t>5840 SW 71st Street, B</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>South Miami</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -1897,18 +1897,16 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>33130</t>
+          <t>33143</t>
         </is>
       </c>
       <c r="I30" s="7" t="n">
         <v>46178</v>
       </c>
-      <c r="J30" s="7" t="n">
-        <v>46477</v>
-      </c>
+      <c r="J30" s="6" t="inlineStr"/>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>Lucky 9 Bartending &amp; Consulting INC</t>
+          <t>La Traila BBQ LLC</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1961,7 +1959,7 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -1971,7 +1969,7 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -1999,26 +1997,16 @@
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>Catering</t>
+          <t>Full liquor (quota), on/off premises</t>
         </is>
       </c>
       <c r="B10" s="16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t>Full liquor (quota), on/off premises</t>
-        </is>
-      </c>
-      <c r="B11" s="16" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>